<commit_message>
change font across all sheets
</commit_message>
<xml_diff>
--- a/Excel/Common_v03.xlsx
+++ b/Excel/Common_v03.xlsx
@@ -736,108 +736,106 @@
   </numFmts>
   <fonts count="34" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <i/>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1" tint="0.499984740745262"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1" tint="0.14999847407452621"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1" tint="0.14999847407452621"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <b/>
-      <sz val="20"/>
+      <sz val="18"/>
       <color rgb="FF183C1B"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color rgb="FF183C1B"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <i/>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1" tint="0.34998626667073579"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1" tint="0.34998626667073579"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1" tint="0.14996795556505021"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="20"/>
+      <sz val="18"/>
       <color rgb="FFCC6600"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <i/>
-      <sz val="12"/>
+      <sz val="10"/>
       <color rgb="FFCC6600"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color rgb="FF533001"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <i/>
       <strike/>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1" tint="0.499984740745262"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <b/>
       <i/>
       <strike/>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1" tint="0.499984740745262"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
@@ -848,114 +846,112 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="14"/>
       <color theme="0"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1" tint="0.249977111117893"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1" tint="0.499984740745262"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="0" tint="-4.9989318521683403E-2"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1" tint="0.34998626667073579"/>
-      <name val="Times New Roman"/>
+      <color theme="0"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1" tint="0.499984740745262"/>
+      <name val="Arial"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0" tint="-4.9989318521683403E-2"/>
+      <name val="Arial"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1" tint="0.34998626667073579"/>
+      <name val="Arial"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="18"/>
+      <sz val="16"/>
       <color theme="1" tint="0.14996795556505021"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1" tint="0.34998626667073579"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="5"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1" tint="0.34998626667073579"/>
-      <name val="Times New Roman"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="5"/>
-      <name val="Times New Roman"/>
+      <color theme="1" tint="0.24994659260841701"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1" tint="0.24994659260841701"/>
-      <name val="Times New Roman"/>
+      <sz val="10"/>
+      <color rgb="FFC44340"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FFC44340"/>
-      <name val="Times New Roman"/>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF008000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="10"/>
       <color rgb="FF0070C0"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="0" tint="-0.499984740745262"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="9"/>
       <color theme="0" tint="-0.499984740745262"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="10"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF404040"/>
-      <name val="Times New Roman"/>
+      <name val="Arial"/>
       <family val="1"/>
     </font>
   </fonts>
@@ -1387,11 +1383,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1411,11 +1406,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1435,11 +1429,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1459,11 +1452,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1483,11 +1475,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1507,11 +1498,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1531,11 +1521,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1555,11 +1544,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1579,11 +1567,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1603,11 +1590,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1627,11 +1613,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1651,11 +1636,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1675,11 +1659,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1699,11 +1682,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1723,11 +1705,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1747,11 +1728,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1771,11 +1751,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1795,11 +1774,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1819,11 +1797,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1843,11 +1820,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1867,11 +1843,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1891,11 +1866,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1915,11 +1889,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1939,11 +1912,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1963,11 +1935,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -1987,11 +1958,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2011,11 +1981,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2035,11 +2004,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2059,11 +2027,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2083,11 +2050,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2107,11 +2073,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2131,11 +2096,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2155,11 +2119,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2179,11 +2142,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2203,11 +2165,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2227,11 +2188,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2251,11 +2211,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2275,11 +2234,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2299,11 +2257,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2323,11 +2280,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -2347,11 +2303,10 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Times New Roman"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="none">
@@ -3241,12 +3196,12 @@
     </a:clrScheme>
     <a:fontScheme name="Custom 1">
       <a:majorFont>
-        <a:latin typeface="Times New Roman"/>
+        <a:latin typeface="Arial"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Times New Roman"/>
+        <a:latin typeface="Arial"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -3457,31 +3412,31 @@
     <tabColor rgb="FF0C769E"/>
   </sheetPr>
   <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="20" x14ac:dyDescent="0.25" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25" ht="30" customHeight="1">
       <c r="A1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="A3" s="15" t="str">
         <f>HYPERLINK("#'Home'!A1", "Home")</f>
         <v>Home</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="A6" s="16" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="20" x14ac:dyDescent="0.25" customHeight="1">
       <c r="A7" s="17" t="str">
         <f>HYPERLINK("#'Constants - Common'!A1", "Constants - Common")</f>
         <v>Constants - Common</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" ht="20" x14ac:dyDescent="0.25" customHeight="1">
       <c r="A8" s="17" t="str">
         <f>HYPERLINK("#'Acknowledgements'!A1", "Acknowledgements")</f>
         <v>Acknowledgements</v>
@@ -3498,7 +3453,7 @@
     <tabColor theme="2" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:BY297"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20" x14ac:dyDescent="0.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="30.7109375" style="6" customWidth="1"/>
     <col min="2" max="2" width="2.7109375" style="6" customWidth="1"/>
@@ -3531,10 +3486,10 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:65" s="8" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:65" s="8" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2"/>
     </row>
-    <row r="3" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="str">
         <f>HYPERLINK("#'Home'!A1", "Home")</f>
         <v>Home</v>
@@ -3561,11 +3516,11 @@
       <c r="V3" s="9"/>
       <c r="W3" s="9"/>
     </row>
-    <row r="4" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4"/>
       <c r="BM4" s="2"/>
     </row>
-    <row r="5" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5"/>
       <c r="D5" s="5" t="str" cm="1">
         <f t="array" ref="D5">Common_SourceData.Common_SourceData_AustralianStatesTerritories_Title()</f>
@@ -3573,7 +3528,7 @@
       </c>
       <c r="BM5" s="2"/>
     </row>
-    <row r="6" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>68</v>
       </c>
@@ -3587,7 +3542,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="str">
         <f>HYPERLINK("#'Constants - Common'!A1", "Constants - Common")</f>
         <v>Constants - Common</v>
@@ -3605,7 +3560,7 @@
         <v>NSW</v>
       </c>
     </row>
-    <row r="8" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="str">
         <f>HYPERLINK("#'Acknowledgements'!A1", "Acknowledgements")</f>
         <v>Acknowledgements</v>
@@ -3623,7 +3578,7 @@
         <v>ACT</v>
       </c>
     </row>
-    <row r="9" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9"/>
       <c r="D9" s="11" t="str" cm="1">
         <f t="array" ref="D9">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</f>
@@ -3638,7 +3593,7 @@
         <v>VIC</v>
       </c>
     </row>
-    <row r="10" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10"/>
       <c r="D10" s="11" t="str" cm="1">
         <f t="array" ref="D10">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</f>
@@ -3653,7 +3608,7 @@
         <v>QLD</v>
       </c>
     </row>
-    <row r="11" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11"/>
       <c r="D11" s="11" t="str" cm="1">
         <f t="array" ref="D11">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</f>
@@ -3669,7 +3624,7 @@
       </c>
       <c r="BM11" s="2"/>
     </row>
-    <row r="12" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12"/>
       <c r="D12" s="11" t="str" cm="1">
         <f t="array" ref="D12">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</f>
@@ -3685,7 +3640,7 @@
       </c>
       <c r="BM12" s="2"/>
     </row>
-    <row r="13" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13"/>
       <c r="D13" s="11" t="str" cm="1">
         <f t="array" ref="D13">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</f>
@@ -3700,7 +3655,7 @@
         <v>TAS</v>
       </c>
     </row>
-    <row r="14" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14"/>
       <c r="D14" s="11" t="str" cm="1">
         <f t="array" ref="D14">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</f>
@@ -3715,129 +3670,129 @@
         <v>NT</v>
       </c>
     </row>
-    <row r="15" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15"/>
     </row>
-    <row r="16" spans="1:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:65" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16"/>
     </row>
-    <row r="17" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17"/>
     </row>
-    <row r="18" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18"/>
       <c r="D18" s="5" t="str" cm="1">
         <f t="array" ref="D18">Common_SourceData.Common_SourceData_WASA4Areas_Title()</f>
         <v>ABS Statistcal Areas Level 4 - Western Australia</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19"/>
       <c r="D19" s="4" t="str" cm="1">
         <f t="array" ref="D19">Common_SourceData.Common_SourceData_WASA4Areas_Source()</f>
         <v>Australian Bureau of Statistics (ABS) - Statistical Areas Level 2 - 2021 - Shapefile</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20"/>
       <c r="D20" s="11" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21"/>
       <c r="D21" s="11" t="str" cm="1">
         <f t="array" ref="D21">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Bunbury</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22"/>
       <c r="D22" s="11" t="str" cm="1">
         <f t="array" ref="D22">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Mandurah</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23"/>
       <c r="D23" s="11" t="str" cm="1">
         <f t="array" ref="D23">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Perth - Inner</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24"/>
       <c r="D24" s="11" t="str" cm="1">
         <f t="array" ref="D24">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Perth - North East</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25"/>
       <c r="D25" s="11" t="str" cm="1">
         <f t="array" ref="D25">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Perth - North West</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26"/>
       <c r="D26" s="11" t="str" cm="1">
         <f t="array" ref="D26">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Perth - South East</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27"/>
       <c r="D27" s="11" t="str" cm="1">
         <f t="array" ref="D27">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Perth - South West</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28"/>
       <c r="D28" s="11" t="str" cm="1">
         <f t="array" ref="D28">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Western Australia - Wheat Belt</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29"/>
       <c r="D29" s="11" t="str" cm="1">
         <f t="array" ref="D29">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Western Australia - Outback (North)</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30"/>
       <c r="D30" s="11" t="str" cm="1">
         <f t="array" ref="D30">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</f>
         <v>Western Australia - Outback (South)</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31"/>
     </row>
-    <row r="32" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32"/>
     </row>
-    <row r="33" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33"/>
     </row>
-    <row r="34" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34"/>
       <c r="D34" s="5" t="str" cm="1">
         <f t="array" ref="D34">Common_SourceData.Common_SourceData_GWP_Title()</f>
         <v>Global warming potential for greenhouse gases</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35"/>
       <c r="D35" s="4" t="str" cm="1">
         <f t="array" ref="D35">Common_SourceData.Common_SourceData_GWP_Source()</f>
         <v>XXXXXXX</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36"/>
       <c r="D36" s="11" t="s">
         <v>5</v>
@@ -3846,7 +3801,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37"/>
       <c r="D37" s="11" t="str" cm="1">
         <f t="array" ref="D37">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</f>
@@ -3857,7 +3812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38"/>
       <c r="D38" s="11" t="str" cm="1">
         <f t="array" ref="D38">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</f>
@@ -3868,7 +3823,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39"/>
       <c r="D39" s="11" t="str" cm="1">
         <f t="array" ref="D39">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</f>
@@ -3879,7 +3834,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40"/>
       <c r="D40" s="11" t="str" cm="1">
         <f t="array" ref="D40">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</f>
@@ -3890,7 +3845,7 @@
         <v>6630</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41"/>
       <c r="D41" s="11" t="str" cm="1">
         <f t="array" ref="D41">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</f>
@@ -3901,7 +3856,7 @@
         <v>12200</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42"/>
       <c r="D42" s="11" t="str" cm="1">
         <f t="array" ref="D42">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</f>
@@ -3912,7 +3867,7 @@
         <v>22800</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43"/>
       <c r="D43" s="11" t="str" cm="1">
         <f t="array" ref="D43">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</f>
@@ -3923,24 +3878,24 @@
         <v>17200</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44"/>
     </row>
-    <row r="45" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45"/>
       <c r="D45" s="5" t="str" cm="1">
         <f t="array" ref="D45">Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Title()</f>
         <v>Factor to convert elemental mass of gas to molecular mass</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46"/>
       <c r="D46" s="4" t="str" cm="1">
         <f t="array" ref="D46">Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Source()</f>
         <v>XXXXXXX</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47"/>
       <c r="D47" s="11" t="s">
         <v>5</v>
@@ -3958,7 +3913,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48"/>
       <c r="D48" s="11" t="str" cm="1">
         <f t="array" ref="D48">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
@@ -3981,7 +3936,7 @@
         <v>3.6666666666666665</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49"/>
       <c r="D49" s="11" t="str" cm="1">
         <f t="array" ref="D49">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
@@ -4004,7 +3959,7 @@
         <v>1.3333333333333333</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50"/>
       <c r="D50" s="11" t="str" cm="1">
         <f t="array" ref="D50">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
@@ -4027,7 +3982,7 @@
         <v>1.5714285714285714</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51"/>
       <c r="D51" s="11" t="str" cm="1">
         <f t="array" ref="D51">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
@@ -4050,7 +4005,7 @@
         <v>3.2857142857142856</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52"/>
       <c r="D52" s="11" t="str" cm="1">
         <f t="array" ref="D52">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
@@ -4073,7 +4028,7 @@
         <v>2.3333333333333335</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53"/>
       <c r="D53" s="11" t="str" cm="1">
         <f t="array" ref="D53">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
@@ -4096,7 +4051,7 @@
         <v>3.6666666666666665</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54"/>
       <c r="D54" s="11" t="str" cm="1">
         <f t="array" ref="D54">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</f>
@@ -4119,49 +4074,49 @@
         <v>1.1666666666666667</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55"/>
     </row>
-    <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56"/>
     </row>
-    <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57"/>
       <c r="D57" s="5" t="str" cm="1">
         <f t="array" ref="D57">Common_SourceData.Common_SourceData_WetAndDryZones_Title()</f>
         <v>VEERG Australian wet and dry zones</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58"/>
       <c r="D58" s="4" t="str" cm="1">
         <f t="array" ref="D58">Common_SourceData.Common_SourceData_WetAndDryZones_Source()</f>
         <v>VEERG 2026: Table 1.2: Translating climate zones to wet and dry zones</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59"/>
       <c r="D59" s="13" t="str" cm="1">
         <f t="array" ref="D59:D61">"⚠️" &amp; Common_SourceData.Common_SourceData_WetAndDryZones_Variation()</f>
         <v>⚠️VARIATION OF SOURCE DATA:</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60"/>
       <c r="D60" s="13" t="str">
         <v>⚠️Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61"/>
       <c r="D61" s="13" t="str">
         <v>⚠️Fixed typo - Changed 'Fry' to 'Dry'.</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62"/>
     </row>
-    <row r="63" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63"/>
       <c r="D63" s="11" t="s">
         <v>0</v>
@@ -4170,7 +4125,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64"/>
       <c r="D64" s="11" t="str" cm="1">
         <f t="array" ref="D64">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4181,7 +4136,7 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65"/>
       <c r="D65" s="11" t="str" cm="1">
         <f t="array" ref="D65">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4192,7 +4147,7 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66"/>
       <c r="D66" s="11" t="str" cm="1">
         <f t="array" ref="D66">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4203,7 +4158,7 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67"/>
       <c r="D67" s="11" t="str" cm="1">
         <f t="array" ref="D67">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4214,7 +4169,7 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68"/>
       <c r="D68" s="11" t="str" cm="1">
         <f t="array" ref="D68">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4225,7 +4180,7 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69"/>
       <c r="D69" s="11" t="str" cm="1">
         <f t="array" ref="D69">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4236,7 +4191,7 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70"/>
       <c r="D70" s="11" t="str" cm="1">
         <f t="array" ref="D70">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4247,7 +4202,7 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71"/>
       <c r="D71" s="11" t="str" cm="1">
         <f t="array" ref="D71">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4258,7 +4213,7 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72"/>
       <c r="D72" s="11" t="str" cm="1">
         <f t="array" ref="D72">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4269,7 +4224,7 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73"/>
       <c r="D73" s="11" t="str" cm="1">
         <f t="array" ref="D73">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4280,7 +4235,7 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74"/>
       <c r="D74" s="11" t="str" cm="1">
         <f t="array" ref="D74">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4291,7 +4246,7 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75"/>
       <c r="D75" s="11" t="str" cm="1">
         <f t="array" ref="D75">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4302,7 +4257,7 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="76" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76"/>
       <c r="D76" s="11" t="str" cm="1">
         <f t="array" ref="D76">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4313,7 +4268,7 @@
         <v>Wet climate zone</v>
       </c>
     </row>
-    <row r="77" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77"/>
       <c r="D77" s="11" t="str" cm="1">
         <f t="array" ref="D77">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</f>
@@ -4324,64 +4279,64 @@
         <v>Dry climate zone</v>
       </c>
     </row>
-    <row r="78" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78"/>
     </row>
-    <row r="79" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79"/>
     </row>
-    <row r="80" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80"/>
     </row>
-    <row r="81" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81"/>
       <c r="D81" s="5" t="str" cm="1">
         <f t="array" ref="D81">Common_SourceData.Common_SourceData_ClimateZones_Title()</f>
         <v>VEERG Australian climate zones</v>
       </c>
     </row>
-    <row r="82" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82"/>
       <c r="D82" s="4" t="str" cm="1">
         <f t="array" ref="D82">Common_SourceData.Common_SourceData_ClimateZones_Source()</f>
         <v>VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions</v>
       </c>
     </row>
-    <row r="83" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83"/>
       <c r="D83" s="13" t="str" cm="1">
         <f t="array" ref="D83:D87">"⚠️" &amp; Common_SourceData.Common_SourceData_ClimateZones_Variation()</f>
         <v>⚠️VARIATION OF SOURCE DATA:</v>
       </c>
     </row>
-    <row r="84" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84"/>
       <c r="D84" s="13" t="str">
         <v>⚠️Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.</v>
       </c>
     </row>
-    <row r="85" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85"/>
       <c r="D85" s="13" t="str">
         <v>⚠️Fixed typo in MAT value for warm temperate dry - changed 10 to 11.</v>
       </c>
     </row>
-    <row r="86" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86"/>
       <c r="D86" s="13" t="str">
         <v>⚠️Added min and max columns for MAT, MAP, frost days per year, elevation, MAP:PET to calculate zones from real climate data.</v>
       </c>
     </row>
-    <row r="87" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87"/>
       <c r="D87" s="13" t="str">
         <v>⚠️GAF accepts rainfall as a proxy for precipitation.</v>
       </c>
     </row>
-    <row r="88" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88"/>
     </row>
-    <row r="89" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89"/>
       <c r="D89" s="11" t="s">
         <v>0</v>
@@ -4433,7 +4388,7 @@
       </c>
       <c r="T89" s="11"/>
     </row>
-    <row r="90" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90"/>
       <c r="D90" s="11" t="str" cm="1">
         <f t="array" ref="D90">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
@@ -4501,7 +4456,7 @@
       </c>
       <c r="T90" s="11"/>
     </row>
-    <row r="91" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91"/>
       <c r="D91" s="11" t="str" cm="1">
         <f t="array" ref="D91">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
@@ -4569,7 +4524,7 @@
       </c>
       <c r="T91" s="11"/>
     </row>
-    <row r="92" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92"/>
       <c r="D92" s="11" t="str" cm="1">
         <f t="array" ref="D92">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
@@ -4637,7 +4592,7 @@
       </c>
       <c r="T92" s="11"/>
     </row>
-    <row r="93" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93"/>
       <c r="D93" s="11" t="str" cm="1">
         <f t="array" ref="D93">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
@@ -4705,7 +4660,7 @@
       </c>
       <c r="T93" s="11"/>
     </row>
-    <row r="94" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94"/>
       <c r="D94" s="11" t="str" cm="1">
         <f t="array" ref="D94">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
@@ -4773,7 +4728,7 @@
       </c>
       <c r="T94" s="11"/>
     </row>
-    <row r="95" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95"/>
       <c r="D95" s="11" t="str" cm="1">
         <f t="array" ref="D95">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
@@ -4841,7 +4796,7 @@
       </c>
       <c r="T95" s="11"/>
     </row>
-    <row r="96" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96"/>
       <c r="D96" s="11" t="str" cm="1">
         <f t="array" ref="D96">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
@@ -4909,7 +4864,7 @@
       </c>
       <c r="T96" s="11"/>
     </row>
-    <row r="97" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97"/>
       <c r="D97" s="11" t="str" cm="1">
         <f t="array" ref="D97">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</f>
@@ -4977,66 +4932,66 @@
       </c>
       <c r="T97" s="11"/>
     </row>
-    <row r="98" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98"/>
     </row>
-    <row r="99" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99"/>
       <c r="D99" s="12" t="str" cm="1">
         <f t="array" ref="D99:D102">Common_SourceData.Common_SourceData_ClimateZones_Appendices()</f>
         <v>Note:</v>
       </c>
     </row>
-    <row r="100" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100"/>
       <c r="D100" s="12" t="str">
         <v>MAT = mean annual temperature</v>
       </c>
     </row>
-    <row r="101" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101"/>
       <c r="D101" s="12" t="str">
         <v>MAP = mean annual precipitation</v>
       </c>
     </row>
-    <row r="102" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102"/>
       <c r="D102" s="12" t="str">
         <v>PET = potential evapotranspiration</v>
       </c>
     </row>
-    <row r="103" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103"/>
       <c r="D103" s="12"/>
     </row>
-    <row r="104" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104"/>
     </row>
-    <row r="105" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105"/>
       <c r="D105" s="5" t="str" cm="1">
         <f t="array" ref="D105">Common_SourceData.Common_SourceData_TemperatureZones_Title()</f>
         <v>VEERG Australian temperature zones</v>
       </c>
     </row>
-    <row r="106" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106"/>
       <c r="D106" s="4" t="str" cm="1">
         <f t="array" ref="D106">Common_SourceData.Common_SourceData_TemperatureZones_Source()</f>
         <v>VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions</v>
       </c>
     </row>
-    <row r="107" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107"/>
       <c r="D107" s="13" t="str" cm="1">
         <f t="array" ref="D107">"⚠️" &amp; Common_SourceData.Common_SourceData_TemperatureZones_Variation()</f>
         <v>⚠️VARIATION OF SOURCE DATA: Added extra MAT min and MAT max columns to calculate zone from real temperature data.</v>
       </c>
     </row>
-    <row r="108" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108"/>
     </row>
-    <row r="109" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109"/>
       <c r="D109" s="11" t="s">
         <v>27</v>
@@ -5051,7 +5006,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="110" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110"/>
       <c r="D110" s="11" t="str" cm="1">
         <f t="array" ref="D110">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</f>
@@ -5070,7 +5025,7 @@
         <v>999999</v>
       </c>
     </row>
-    <row r="111" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111"/>
       <c r="D111" s="11" t="str" cm="1">
         <f t="array" ref="D111">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</f>
@@ -5089,7 +5044,7 @@
         <v>25.998999999999999</v>
       </c>
     </row>
-    <row r="112" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112"/>
       <c r="D112" s="11" t="str" cm="1">
         <f t="array" ref="D112">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</f>
@@ -5108,13 +5063,13 @@
         <v>14.999000000000001</v>
       </c>
     </row>
-    <row r="113" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113"/>
     </row>
-    <row r="114" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114"/>
     </row>
-    <row r="115" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115"/>
       <c r="D115" s="5" t="str" cm="1">
         <f t="array" ref="D115">Common_SourceData.Common_SourceData_RainfallZones_Title()</f>
@@ -5122,7 +5077,7 @@
       </c>
       <c r="BN115" s="6"/>
     </row>
-    <row r="116" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116"/>
       <c r="D116" s="4" t="str" cm="1">
         <f t="array" ref="D116">Common_SourceData.Common_SourceData_RainfallZones_Source()</f>
@@ -5130,7 +5085,7 @@
       </c>
       <c r="BN116" s="6"/>
     </row>
-    <row r="117" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117"/>
       <c r="D117" s="13" t="str" cm="1">
         <f t="array" ref="D117">"⚠️" &amp; Common_SourceData.Common_SourceData_RainfallZones_Variation()</f>
@@ -5138,11 +5093,11 @@
       </c>
       <c r="BN117" s="6"/>
     </row>
-    <row r="118" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118"/>
       <c r="BN118" s="6"/>
     </row>
-    <row r="119" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119"/>
       <c r="D119" s="11" t="s">
         <v>30</v>
@@ -5158,7 +5113,7 @@
       </c>
       <c r="BN119" s="6"/>
     </row>
-    <row r="120" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120"/>
       <c r="D120" s="11" t="str" cm="1">
         <f t="array" ref="D120">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</f>
@@ -5178,7 +5133,7 @@
       </c>
       <c r="BN120" s="6"/>
     </row>
-    <row r="121" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121"/>
       <c r="D121" s="11" t="str" cm="1">
         <f t="array" ref="D121">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</f>
@@ -5198,31 +5153,31 @@
       </c>
       <c r="BN121" s="6"/>
     </row>
-    <row r="122" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122"/>
       <c r="BN122" s="6"/>
     </row>
-    <row r="123" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123"/>
     </row>
-    <row r="124" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124"/>
       <c r="D124" s="5" t="str" cm="1">
         <f t="array" ref="D124">Common_SourceData.Common_SourceData_LeachingZones_Title()</f>
         <v>VEERG Australian leaching zones</v>
       </c>
     </row>
-    <row r="125" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125"/>
       <c r="D125" s="4" t="str" cm="1">
         <f t="array" ref="D125">Common_SourceData.Common_SourceData_LeachingZones_Source()</f>
         <v>VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions</v>
       </c>
     </row>
-    <row r="126" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126"/>
     </row>
-    <row r="127" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127"/>
       <c r="D127" s="11" t="s">
         <v>32</v>
@@ -5231,7 +5186,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="128" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128"/>
       <c r="D128" s="11" t="str" cm="1">
         <f t="array" ref="D128">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</f>
@@ -5242,7 +5197,7 @@
         <v>Σ(𝑟𝑎𝑖𝑛)&gt;Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦</v>
       </c>
     </row>
-    <row r="129" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129"/>
       <c r="D129" s="11" t="str" cm="1">
         <f t="array" ref="D129">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</f>
@@ -5253,13 +5208,13 @@
         <v>Σ(𝑟𝑎𝑖𝑛)≤Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦</v>
       </c>
     </row>
-    <row r="130" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130"/>
     </row>
-    <row r="131" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131"/>
     </row>
-    <row r="132" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132"/>
       <c r="D132" s="5" t="str" cm="1">
         <f t="array" ref="D132">Common_SourceData.Common_SourceData_FracWET_Title()</f>
@@ -5267,7 +5222,7 @@
       </c>
       <c r="E132" s="10"/>
     </row>
-    <row r="133" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133"/>
       <c r="D133" s="4" t="str" cm="1">
         <f t="array" ref="D133">Common_SourceData.Common_SourceData_FracWET_Source()</f>
@@ -5275,7 +5230,7 @@
       </c>
       <c r="E133" s="10"/>
     </row>
-    <row r="134" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134"/>
       <c r="D134" t="s">
         <v>37</v>
@@ -5284,7 +5239,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="135" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135"/>
       <c r="D135" t="str" cm="1">
         <f t="array" ref="D135">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</f>
@@ -5295,7 +5250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136"/>
       <c r="D136" s="1" t="str" cm="1">
         <f t="array" ref="D136">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</f>
@@ -5306,10 +5261,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137"/>
     </row>
-    <row r="138" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138"/>
       <c r="BN138" s="6"/>
       <c r="BO138" s="6"/>
@@ -5324,7 +5279,7 @@
       <c r="BX138" s="6"/>
       <c r="BY138" s="6"/>
     </row>
-    <row r="139" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139"/>
       <c r="D139" s="5" t="str" cm="1">
         <f t="array" ref="D139">Common_SourceData.Common_SourceData_FracWETIrrigation_Title()</f>
@@ -5343,7 +5298,7 @@
       <c r="BX139" s="6"/>
       <c r="BY139" s="6"/>
     </row>
-    <row r="140" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140"/>
       <c r="D140" s="4" t="str" cm="1">
         <f t="array" ref="D140">Common_SourceData.Common_SourceData_FracWETIrrigation_Source()</f>
@@ -5362,7 +5317,7 @@
       <c r="BX140" s="6"/>
       <c r="BY140" s="6"/>
     </row>
-    <row r="141" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141"/>
       <c r="D141" s="13" t="str" cm="1">
         <f t="array" ref="D141">Common_SourceData.Common_SourceData_FracWETIrrigation_Variation()</f>
@@ -5370,7 +5325,7 @@
       </c>
       <c r="BN141" s="6"/>
     </row>
-    <row r="142" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142"/>
       <c r="D142" s="11" t="s">
         <v>46</v>
@@ -5380,7 +5335,7 @@
       </c>
       <c r="BN142" s="6"/>
     </row>
-    <row r="143" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143"/>
       <c r="D143" s="11" t="str" cm="1">
         <f t="array" ref="D143">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
@@ -5392,7 +5347,7 @@
       </c>
       <c r="BN143" s="6"/>
     </row>
-    <row r="144" spans="1:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:77" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144"/>
       <c r="D144" s="1" t="str" cm="1">
         <f t="array" ref="D144">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
@@ -5404,7 +5359,7 @@
       </c>
       <c r="BN144" s="6"/>
     </row>
-    <row r="145" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145"/>
       <c r="D145" s="1" t="str" cm="1">
         <f t="array" ref="D145">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
@@ -5416,7 +5371,7 @@
       </c>
       <c r="BN145" s="6"/>
     </row>
-    <row r="146" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146"/>
       <c r="D146" s="1" t="str" cm="1">
         <f t="array" ref="D146">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
@@ -5428,7 +5383,7 @@
       </c>
       <c r="BN146" s="6"/>
     </row>
-    <row r="147" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147"/>
       <c r="D147" s="1" t="str" cm="1">
         <f t="array" ref="D147">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</f>
@@ -5440,15 +5395,15 @@
       </c>
       <c r="BN147" s="6"/>
     </row>
-    <row r="148" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148"/>
       <c r="BN148" s="6"/>
     </row>
-    <row r="149" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149"/>
       <c r="BN149" s="6"/>
     </row>
-    <row r="150" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150"/>
       <c r="D150" s="5" t="str" cm="1">
         <f t="array" ref="D150">Common_SourceData.Common_SourceData_DataScores_Scope3_Title()</f>
@@ -5456,7 +5411,7 @@
       </c>
       <c r="BN150" s="6"/>
     </row>
-    <row r="151" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151"/>
       <c r="D151" s="4" t="str" cm="1">
         <f t="array" ref="D151">Common_SourceData.Common_SourceData_DataScores_Scope3_Source()</f>
@@ -5464,11 +5419,11 @@
       </c>
       <c r="BN151" s="6"/>
     </row>
-    <row r="152" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152"/>
       <c r="BN152" s="6"/>
     </row>
-    <row r="153" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153"/>
       <c r="D153" s="11" t="s">
         <v>34</v>
@@ -5488,7 +5443,7 @@
       <c r="BL153" s="2"/>
       <c r="BM153" s="2"/>
     </row>
-    <row r="154" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154"/>
       <c r="D154" s="11" t="str" cm="1">
         <f t="array" ref="D154">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
@@ -5510,7 +5465,7 @@
       <c r="BL154" s="2"/>
       <c r="BM154" s="2"/>
     </row>
-    <row r="155" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155"/>
       <c r="D155" s="11" t="str" cm="1">
         <f t="array" ref="D155">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
@@ -5532,7 +5487,7 @@
       <c r="BL155" s="2"/>
       <c r="BM155" s="2"/>
     </row>
-    <row r="156" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156"/>
       <c r="D156" s="11" t="str" cm="1">
         <f t="array" ref="D156">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
@@ -5543,7 +5498,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="157" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157"/>
       <c r="D157" s="11" t="str" cm="1">
         <f t="array" ref="D157">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
@@ -5554,7 +5509,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="158" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158"/>
       <c r="D158" s="11" t="str" cm="1">
         <f t="array" ref="D158">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
@@ -5565,34 +5520,34 @@
         <v>5</v>
       </c>
     </row>
-    <row r="159" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159"/>
     </row>
-    <row r="160" spans="1:66" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:66" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160"/>
     </row>
-    <row r="161" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D161" s="5" t="str" cm="1">
         <f t="array" ref="D161">Common_SourceData.Common_SourceData_FracLEACH_Title()</f>
         <v>Fraction of N that is available for leaching and runoff</v>
       </c>
       <c r="E161" s="10"/>
     </row>
-    <row r="162" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D162" s="4" t="str" cm="1">
         <f t="array" ref="D162">Common_SourceData.Common_SourceData_FracLEACH_Source()</f>
         <v>VEERG 2026:5.5.2.3 Constant Parameters</v>
       </c>
       <c r="E162" s="10"/>
     </row>
-    <row r="163" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D163" s="4" t="str" cm="1">
         <f t="array" ref="D163">Common_SourceData.Common_SourceData_FracLEACH_NIRReference()</f>
         <v>National Inventory Report Volume 1: Leaching and runoff (3.D.b.2)</v>
       </c>
       <c r="E163" s="10"/>
     </row>
-    <row r="164" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D164" s="10" t="str" cm="1">
         <f t="array" ref="D164:E164">Common_SourceData.Common_SourceData_FracLEACH_Data()</f>
         <v>FracLEACH</v>
@@ -5601,17 +5556,17 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="165" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BN165" s="6"/>
       <c r="BO165" s="6"/>
       <c r="BP165" s="6"/>
     </row>
-    <row r="166" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BN166" s="6"/>
       <c r="BO166" s="6"/>
       <c r="BP166" s="6"/>
     </row>
-    <row r="167" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D167" s="5" t="str" cm="1">
         <f t="array" ref="D167">Common_SourceData.Common_SourceData_EFleach_Title()</f>
         <v>Emission factor for nitrogen leaching and runoff</v>
@@ -5620,7 +5575,7 @@
       <c r="BO167" s="6"/>
       <c r="BP167" s="6"/>
     </row>
-    <row r="168" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D168" s="4" t="str" cm="1">
         <f t="array" ref="D168">Common_SourceData.Common_SourceData_EFleach_Source()</f>
         <v>VEERG 2026:5.5.2.3 Constant Parameters</v>
@@ -5629,7 +5584,7 @@
       <c r="BO168" s="6"/>
       <c r="BP168" s="6"/>
     </row>
-    <row r="169" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D169" s="4" t="str" cm="1">
         <f t="array" ref="D169">Common_SourceData.Common_SourceData_EFleach_NIRReference()</f>
         <v>National Inventory Report Volume 1: Equation 3.D.B_10</v>
@@ -5638,7 +5593,7 @@
       <c r="BO169" s="6"/>
       <c r="BP169" s="6"/>
     </row>
-    <row r="170" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D170" s="1" t="str" cm="1">
         <f t="array" ref="D170:E170">Common_SourceData.Common_SourceData_EFleach_Data()</f>
         <v>EFleach</v>
@@ -5650,17 +5605,17 @@
       <c r="BO170" s="6"/>
       <c r="BP170" s="6"/>
     </row>
-    <row r="171" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BN171" s="6"/>
       <c r="BO171" s="6"/>
       <c r="BP171" s="6"/>
     </row>
-    <row r="172" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BN172" s="6"/>
       <c r="BO172" s="6"/>
       <c r="BP172" s="6"/>
     </row>
-    <row r="173" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D173" s="5" t="str" cm="1">
         <f t="array" ref="D173">Common_SourceData.Common_SourceData_DensityOfMethane_Title()</f>
         <v>p = density of methane</v>
@@ -5669,7 +5624,7 @@
       <c r="BO173" s="6"/>
       <c r="BP173" s="6"/>
     </row>
-    <row r="174" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D174" s="4" t="str" cm="1">
         <f t="array" ref="D174">Common_SourceData.Common_SourceData_DensityOfMethane_Source()</f>
         <v>National Inventory Report 2023 Volume 1: Equations 3.B.1a_2, 3.B.1c_2, 3.B.3_1, 3.B.4g_2</v>
@@ -5678,7 +5633,7 @@
       <c r="BO174" s="6"/>
       <c r="BP174" s="6"/>
     </row>
-    <row r="175" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D175" s="1" cm="1">
         <f t="array" ref="D175">Common_SourceData.Common_SourceData_DensityOfMethane_Data()</f>
         <v>0.6784</v>
@@ -5691,17 +5646,17 @@
       <c r="BO175" s="6"/>
       <c r="BP175" s="6"/>
     </row>
-    <row r="176" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BN176" s="6"/>
       <c r="BO176" s="6"/>
       <c r="BP176" s="6"/>
     </row>
-    <row r="177" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BN177" s="6"/>
       <c r="BO177" s="6"/>
       <c r="BP177" s="6"/>
     </row>
-    <row r="178" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D178" s="5" t="str" cm="1">
         <f t="array" ref="D178">Common_SourceData.Common_SourceData_EFN2O_Title()</f>
         <v>Nitrous oxide emission factors for inorganic fertiliser application</v>
@@ -5710,7 +5665,7 @@
       <c r="BO178" s="6"/>
       <c r="BP178" s="6"/>
     </row>
-    <row r="179" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D179" s="4" t="str" cm="1">
         <f t="array" ref="D179">Common_SourceData.Common_SourceData_EFN2O_Source()</f>
         <v>VEERG 2026: Table A.2.2.1</v>
@@ -5719,39 +5674,39 @@
       <c r="BO179" s="6"/>
       <c r="BP179" s="6"/>
     </row>
-    <row r="180" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D180" s="12" t="str" cm="1">
         <f t="array" ref="D180">Common_SourceData.Common_SourceData_EFN2O_Unit()</f>
         <v>(kg N2O-N / kg N</v>
       </c>
     </row>
-    <row r="181" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D181" s="13" t="str" cm="1">
         <f t="array" ref="D181:D185">Common_SourceData.Common_SourceData_EFN2O_Variation()</f>
         <v>VARIATION OF SOURCE DATA:</v>
       </c>
     </row>
-    <row r="182" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D182" s="13" t="str">
         <v>Removed duplicate 'Aquaculture' row.</v>
       </c>
     </row>
-    <row r="183" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D183" s="13" t="str">
         <v>Removed asterisks to aid lookup.</v>
       </c>
     </row>
-    <row r="184" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D184" s="13" t="str">
         <v>Added 'production system only', 'rainfall zone' and 'irrigation method' columns to aid lookup.</v>
       </c>
     </row>
-    <row r="185" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D185" s="13" t="str">
         <v>Duplicated 'non-irrigated pasture' row with same EF for low and high rainfall zones to aid lookup.</v>
       </c>
     </row>
-    <row r="186" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D186" s="11" t="s">
         <v>39</v>
       </c>
@@ -5768,7 +5723,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="187" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D187" s="11" t="str" cm="1">
         <f t="array" ref="D187">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Irrigated pasture</v>
@@ -5790,7 +5745,7 @@
         <v>Any</v>
       </c>
     </row>
-    <row r="188" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D188" s="11" t="str" cm="1">
         <f t="array" ref="D188">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Irrigated crop</v>
@@ -5812,7 +5767,7 @@
         <v>Any</v>
       </c>
     </row>
-    <row r="189" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D189" s="11" t="str" cm="1">
         <f t="array" ref="D189">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Non-irrigated pasture</v>
@@ -5834,7 +5789,7 @@
         <v>Low rainfall</v>
       </c>
     </row>
-    <row r="190" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D190" s="11" t="str" cm="1">
         <f t="array" ref="D190">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Non-irrigated pasture</v>
@@ -5856,7 +5811,7 @@
         <v>High rainfall</v>
       </c>
     </row>
-    <row r="191" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D191" s="11" t="str" cm="1">
         <f t="array" ref="D191">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Non-irrigated crop (low rainfall)</v>
@@ -5878,7 +5833,7 @@
         <v>Low rainfall</v>
       </c>
     </row>
-    <row r="192" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="4:68" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D192" s="11" t="str" cm="1">
         <f t="array" ref="D192">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Non-irrigated crop (high rainfall)</v>
@@ -5900,7 +5855,7 @@
         <v>High rainfall</v>
       </c>
     </row>
-    <row r="193" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="4:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D193" s="11" t="str" cm="1">
         <f t="array" ref="D193">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Sugar</v>
@@ -5922,7 +5877,7 @@
         <v>Any</v>
       </c>
     </row>
-    <row r="194" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="4:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D194" s="11" t="str" cm="1">
         <f t="array" ref="D194">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Cotton</v>
@@ -5944,7 +5899,7 @@
         <v>Any</v>
       </c>
     </row>
-    <row r="195" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="4:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D195" s="11" t="str" cm="1">
         <f t="array" ref="D195">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Horticultural crops</v>
@@ -5966,7 +5921,7 @@
         <v>Any</v>
       </c>
     </row>
-    <row r="196" spans="4:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="4:8" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D196" s="11" t="str" cm="1">
         <f t="array" ref="D196">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Rice (continuous flooding)</v>
@@ -5988,7 +5943,7 @@
         <v>Any</v>
       </c>
     </row>
-    <row r="197" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="197" spans="4:8" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D197" s="11" t="str" cm="1">
         <f t="array" ref="D197">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Rice (single and multiple drainage, or alternate wetting and drying)</v>
@@ -6010,7 +5965,7 @@
         <v>Any</v>
       </c>
     </row>
-    <row r="198" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="198" spans="4:8" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D198" s="11" t="str" cm="1">
         <f t="array" ref="D198">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Aquaculture</v>
@@ -6032,7 +5987,7 @@
         <v>Any</v>
       </c>
     </row>
-    <row r="199" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="199" spans="4:8" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D199" s="11" t="str" cm="1">
         <f t="array" ref="D199">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
         <v>Forestry</v>
@@ -6054,31 +6009,31 @@
         <v>Any</v>
       </c>
     </row>
-    <row r="202" spans="4:8" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="202" spans="4:8" ht="20" x14ac:dyDescent="0.25" customHeight="1">
       <c r="D202" s="5" t="str" cm="1">
         <f t="array" ref="D202">Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Title()</f>
         <v>Emission factor for urine and dung deposited on pasture, range or paddock</v>
       </c>
     </row>
-    <row r="203" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="203" spans="4:8" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D203" s="4" t="str" cm="1">
         <f t="array" ref="D203">Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Source()</f>
         <v>VEERG 2026: Table A.2.2.2</v>
       </c>
     </row>
-    <row r="204" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="204" spans="4:8" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D204" s="13" t="str" cm="1">
         <f t="array" ref="D204">Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Variation()</f>
         <v>VARIATION FROM SOURCE DATA: Changed 'Dry climate zones' to singular 'Dry climate zone' to aid lookup.</v>
       </c>
     </row>
-    <row r="205" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="205" spans="4:8" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D205" s="12" t="str" cm="1">
         <f t="array" ref="D205">Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Unit()</f>
         <v>kg N2O - N / kg N</v>
       </c>
     </row>
-    <row r="206" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="206" spans="4:8" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D206" s="11" t="s">
         <v>0</v>
       </c>
@@ -6086,7 +6041,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="207" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="207" spans="4:8" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D207" s="11" t="str" cm="1">
         <f t="array" ref="D207">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</f>
         <v>Wet climate zone</v>
@@ -6096,7 +6051,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="208" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="208" spans="4:8" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D208" s="1" t="str" cm="1">
         <f t="array" ref="D208">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</f>
         <v>Dry climate zone</v>
@@ -6106,13 +6061,13 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="211" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D211" s="1" t="str" cm="1">
         <f t="array" ref="D211">Common_SourceData.Common_SourceData_MonthsToSeasons_Title()</f>
         <v>Months to Seasons Mapping</v>
       </c>
     </row>
-    <row r="212" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D212" s="11" t="s">
         <v>48</v>
       </c>
@@ -6120,7 +6075,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="213" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D213" s="11" t="str" cm="1">
         <f t="array" ref="D213">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>January</v>
@@ -6130,7 +6085,7 @@
         <v>Summer</v>
       </c>
     </row>
-    <row r="214" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D214" s="1" t="str" cm="1">
         <f t="array" ref="D214">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>February</v>
@@ -6140,7 +6095,7 @@
         <v>Summer</v>
       </c>
     </row>
-    <row r="215" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D215" s="1" t="str" cm="1">
         <f t="array" ref="D215">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>March</v>
@@ -6150,7 +6105,7 @@
         <v>Autumn</v>
       </c>
     </row>
-    <row r="216" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D216" s="1" t="str" cm="1">
         <f t="array" ref="D216">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>April</v>
@@ -6160,7 +6115,7 @@
         <v>Autumn</v>
       </c>
     </row>
-    <row r="217" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D217" s="1" t="str" cm="1">
         <f t="array" ref="D217">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>May</v>
@@ -6170,7 +6125,7 @@
         <v>Autumn</v>
       </c>
     </row>
-    <row r="218" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D218" s="1" t="str" cm="1">
         <f t="array" ref="D218">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>June</v>
@@ -6180,7 +6135,7 @@
         <v>Winter</v>
       </c>
     </row>
-    <row r="219" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D219" s="1" t="str" cm="1">
         <f t="array" ref="D219">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>July</v>
@@ -6190,7 +6145,7 @@
         <v>Winter</v>
       </c>
     </row>
-    <row r="220" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D220" s="1" t="str" cm="1">
         <f t="array" ref="D220">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>August</v>
@@ -6200,7 +6155,7 @@
         <v>Winter</v>
       </c>
     </row>
-    <row r="221" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D221" s="1" t="str" cm="1">
         <f t="array" ref="D221">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>September</v>
@@ -6210,7 +6165,7 @@
         <v>Spring</v>
       </c>
     </row>
-    <row r="222" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D222" s="1" t="str" cm="1">
         <f t="array" ref="D222">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>October</v>
@@ -6220,7 +6175,7 @@
         <v>Spring</v>
       </c>
     </row>
-    <row r="223" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D223" s="1" t="str" cm="1">
         <f t="array" ref="D223">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>November</v>
@@ -6230,7 +6185,7 @@
         <v>Spring</v>
       </c>
     </row>
-    <row r="224" spans="4:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="4:5" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D224" s="1" t="str" cm="1">
         <f t="array" ref="D224">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</f>
         <v>December</v>
@@ -6240,25 +6195,25 @@
         <v>Summer</v>
       </c>
     </row>
-    <row r="227" spans="4:19" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="227" spans="4:19" ht="20" x14ac:dyDescent="0.25" customHeight="1">
       <c r="D227" s="5" t="str" cm="1">
         <f t="array" ref="D227">Common_SourceData.Common_SourceData_MCFTemperatureZone_Title()</f>
         <v>Manure Management – Methane conversion factor per temperature zone (fraction) (MCFim)</v>
       </c>
     </row>
-    <row r="228" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="228" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D228" s="4" t="str" cm="1">
         <f t="array" ref="D228">Common_SourceData.Common_SourceData_MCFTemperatureZone_Source()</f>
         <v>VEERG 2026: Table A.1.8.1</v>
       </c>
     </row>
-    <row r="229" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="229" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D229" s="13" t="str" cm="1">
         <f t="array" ref="D229">Common_SourceData.Common_SourceData_MCFTemperatureZone_Variation()</f>
         <v>VARIATION FROM SOURCE: Added row of NIR MMA definitions to aid lookup. Duplicated 'Poultry with and without litter' column with separate NIR definitions to aid lookup. Added 'MAT raw' column to allow lookup of numbers.</v>
       </c>
     </row>
-    <row r="231" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="231" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D231" s="11" t="s">
         <v>50</v>
       </c>
@@ -6308,7 +6263,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="232" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="232" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D232" s="11" t="str" cm="1">
         <f t="array" ref="D232">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Cool</v>
@@ -6374,7 +6329,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="233" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="233" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D233" s="1" t="str" cm="1">
         <f t="array" ref="D233">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Cool</v>
@@ -6440,7 +6395,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="234" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="234" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D234" s="1" t="str" cm="1">
         <f t="array" ref="D234">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Cool</v>
@@ -6506,7 +6461,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="235" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="235" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D235" s="1" t="str" cm="1">
         <f t="array" ref="D235">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Cool</v>
@@ -6572,7 +6527,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="236" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="236" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D236" s="1" t="str" cm="1">
         <f t="array" ref="D236">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Cool</v>
@@ -6638,7 +6593,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="237" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="237" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D237" s="1" t="str" cm="1">
         <f t="array" ref="D237">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -6704,7 +6659,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="238" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="238" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D238" s="1" t="str" cm="1">
         <f t="array" ref="D238">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -6770,7 +6725,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="239" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="239" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D239" s="1" t="str" cm="1">
         <f t="array" ref="D239">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -6836,7 +6791,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="240" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="240" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D240" s="1" t="str" cm="1">
         <f t="array" ref="D240">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -6902,7 +6857,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="241" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="241" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D241" s="1" t="str" cm="1">
         <f t="array" ref="D241">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -6968,7 +6923,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="242" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="242" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D242" s="1" t="str" cm="1">
         <f t="array" ref="D242">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -7034,7 +6989,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="243" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="243" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D243" s="1" t="str" cm="1">
         <f t="array" ref="D243">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -7100,7 +7055,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="244" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="244" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D244" s="1" t="str" cm="1">
         <f t="array" ref="D244">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -7166,7 +7121,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="245" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="245" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D245" s="1" t="str" cm="1">
         <f t="array" ref="D245">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -7232,7 +7187,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="246" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="246" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D246" s="1" t="str" cm="1">
         <f t="array" ref="D246">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -7298,7 +7253,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="247" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="247" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D247" s="1" t="str" cm="1">
         <f t="array" ref="D247">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Temperate</v>
@@ -7364,7 +7319,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="248" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="248" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D248" s="1" t="str" cm="1">
         <f t="array" ref="D248">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Warm</v>
@@ -7430,7 +7385,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="249" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="249" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D249" s="1" t="str" cm="1">
         <f t="array" ref="D249">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Warm</v>
@@ -7496,7 +7451,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="250" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="250" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D250" s="1" t="str" cm="1">
         <f t="array" ref="D250">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</f>
         <v>Warm</v>
@@ -7562,31 +7517,31 @@
         <v>28</v>
       </c>
     </row>
-    <row r="253" spans="4:19" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="253" spans="4:19" ht="20" x14ac:dyDescent="0.25" customHeight="1">
       <c r="D253" s="5" t="str" cm="1">
         <f t="array" ref="D253">Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Title()</f>
         <v>Emission factor for organic fertiliser and crop residues returned to the soil</v>
       </c>
     </row>
-    <row r="254" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="254" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D254" s="4" t="str" cm="1">
         <f t="array" ref="D254">Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Source()</f>
         <v>VEERG 2026: Table A.2.1.4</v>
       </c>
     </row>
-    <row r="255" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="255" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D255" s="1" t="str" cm="1">
         <f t="array" ref="D255">Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Variable()</f>
         <v>EFNi &amp; EFN2Oi</v>
       </c>
     </row>
-    <row r="256" spans="4:19" x14ac:dyDescent="0.25">
+    <row r="256" spans="4:19" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D256" s="12" t="str" cm="1">
         <f t="array" ref="D256">Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Unit()</f>
         <v>kg N2O - N / kg N</v>
       </c>
     </row>
-    <row r="257" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="257" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D257" s="11" t="s">
         <v>66</v>
       </c>
@@ -7594,7 +7549,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="258" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="258" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D258" s="11" t="str" cm="1">
         <f t="array" ref="D258">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</f>
         <v>Wet climate zone</v>
@@ -7604,7 +7559,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="259" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="259" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D259" s="1" t="str" cm="1">
         <f t="array" ref="D259">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</f>
         <v>Dry climate zone</v>
@@ -7614,17 +7569,17 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="263" spans="4:66" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="263" spans="4:66" ht="20" x14ac:dyDescent="0.25" customHeight="1">
       <c r="D263" s="5" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="264" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="264" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D264" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="265" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="265" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D265" s="11" t="s">
         <v>117</v>
       </c>
@@ -7640,7 +7595,7 @@
       <c r="V265" s="1"/>
       <c r="BN265" s="6"/>
     </row>
-    <row r="266" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="266" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D266" s="11" t="s">
         <v>118</v>
       </c>
@@ -7656,7 +7611,7 @@
       <c r="V266" s="1"/>
       <c r="BN266" s="6"/>
     </row>
-    <row r="267" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="267" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D267" s="11" t="s">
         <v>119</v>
       </c>
@@ -7672,7 +7627,7 @@
       <c r="V267" s="1"/>
       <c r="BN267" s="6"/>
     </row>
-    <row r="268" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="268" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D268" s="11" t="s">
         <v>120</v>
       </c>
@@ -7688,7 +7643,7 @@
       <c r="V268" s="1"/>
       <c r="BN268" s="6"/>
     </row>
-    <row r="269" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="269" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D269" s="11" t="s">
         <v>121</v>
       </c>
@@ -7704,7 +7659,7 @@
       <c r="V269" s="1"/>
       <c r="BN269" s="6"/>
     </row>
-    <row r="270" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="270" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D270" s="11" t="s">
         <v>122</v>
       </c>
@@ -7720,12 +7675,12 @@
       <c r="V270" s="1"/>
       <c r="BN270" s="6"/>
     </row>
-    <row r="273" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="273" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D273" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="274" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="274" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D274" s="11" t="s">
         <v>117</v>
       </c>
@@ -7741,7 +7696,7 @@
       <c r="V274" s="1"/>
       <c r="BN274" s="6"/>
     </row>
-    <row r="275" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="275" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D275" s="11" t="s">
         <v>123</v>
       </c>
@@ -7757,7 +7712,7 @@
       <c r="V275" s="1"/>
       <c r="BN275" s="6"/>
     </row>
-    <row r="276" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="276" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D276" s="11" t="s">
         <v>124</v>
       </c>
@@ -7773,7 +7728,7 @@
       <c r="V276" s="1"/>
       <c r="BN276" s="6"/>
     </row>
-    <row r="277" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="277" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D277" s="11" t="s">
         <v>125</v>
       </c>
@@ -7789,7 +7744,7 @@
       <c r="V277" s="1"/>
       <c r="BN277" s="6"/>
     </row>
-    <row r="278" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="278" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D278" s="11" t="s">
         <v>126</v>
       </c>
@@ -7805,7 +7760,7 @@
       <c r="V278" s="1"/>
       <c r="BN278" s="6"/>
     </row>
-    <row r="279" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="279" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D279" s="11" t="s">
         <v>127</v>
       </c>
@@ -7821,12 +7776,12 @@
       <c r="V279" s="1"/>
       <c r="BN279" s="6"/>
     </row>
-    <row r="282" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="282" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D282" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="283" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="283" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D283" s="11" t="s">
         <v>117</v>
       </c>
@@ -7842,7 +7797,7 @@
       <c r="V283" s="1"/>
       <c r="BN283" s="6"/>
     </row>
-    <row r="284" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="284" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D284" s="11" t="s">
         <v>128</v>
       </c>
@@ -7858,7 +7813,7 @@
       <c r="V284" s="1"/>
       <c r="BN284" s="6"/>
     </row>
-    <row r="285" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="285" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D285" s="11" t="s">
         <v>129</v>
       </c>
@@ -7874,7 +7829,7 @@
       <c r="V285" s="1"/>
       <c r="BN285" s="6"/>
     </row>
-    <row r="286" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="286" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D286" s="11" t="s">
         <v>130</v>
       </c>
@@ -7890,7 +7845,7 @@
       <c r="V286" s="1"/>
       <c r="BN286" s="6"/>
     </row>
-    <row r="287" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="287" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D287" s="11" t="s">
         <v>131</v>
       </c>
@@ -7906,7 +7861,7 @@
       <c r="V287" s="1"/>
       <c r="BN287" s="6"/>
     </row>
-    <row r="288" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="288" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D288" s="11" t="s">
         <v>132</v>
       </c>
@@ -7922,12 +7877,12 @@
       <c r="V288" s="1"/>
       <c r="BN288" s="6"/>
     </row>
-    <row r="291" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="291" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D291" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="292" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="292" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D292" s="11" t="s">
         <v>117</v>
       </c>
@@ -7943,7 +7898,7 @@
       <c r="V292" s="1"/>
       <c r="BN292" s="6"/>
     </row>
-    <row r="293" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="293" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D293" s="11" t="s">
         <v>133</v>
       </c>
@@ -7959,7 +7914,7 @@
       <c r="V293" s="1"/>
       <c r="BN293" s="6"/>
     </row>
-    <row r="294" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="294" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D294" s="11" t="s">
         <v>134</v>
       </c>
@@ -7975,7 +7930,7 @@
       <c r="V294" s="1"/>
       <c r="BN294" s="6"/>
     </row>
-    <row r="295" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="295" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D295" s="11" t="s">
         <v>135</v>
       </c>
@@ -7991,7 +7946,7 @@
       <c r="V295" s="1"/>
       <c r="BN295" s="6"/>
     </row>
-    <row r="296" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="296" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D296" s="11" t="s">
         <v>136</v>
       </c>
@@ -8007,7 +7962,7 @@
       <c r="V296" s="1"/>
       <c r="BN296" s="6"/>
     </row>
-    <row r="297" spans="4:66" x14ac:dyDescent="0.25">
+    <row r="297" spans="4:66" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="D297" s="11" t="s">
         <v>137</v>
       </c>
@@ -8058,31 +8013,31 @@
     <tabColor theme="2" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="20" x14ac:dyDescent="0.25" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25" ht="30" customHeight="1">
       <c r="A1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="20" x14ac:dyDescent="0.25" customHeight="1">
       <c r="A3" s="17" t="str">
         <f>HYPERLINK("#'Home'!A1", "Home")</f>
         <v>Home</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25" ht="20" customHeight="1">
       <c r="A6" s="16" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="20" x14ac:dyDescent="0.25" customHeight="1">
       <c r="A7" s="17" t="str">
         <f>HYPERLINK("#'Constants - Common'!A1", "Constants - Common")</f>
         <v>Constants - Common</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" ht="20" x14ac:dyDescent="0.25" customHeight="1">
       <c r="A8" s="18" t="str">
         <f>HYPERLINK("#'Acknowledgements'!A1", "Acknowledgements")</f>
         <v>Acknowledgements</v>

</xml_diff>